<commit_message>
V2 - Mudanças na consulta, usando codigo ibge ao inves de nome
</commit_message>
<xml_diff>
--- a/Cliente.xlsx
+++ b/Cliente.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source\MunicipiosHomologados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AD462D-8738-46CF-AAFE-58D73022CC95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61568E3E-FA53-4723-89FF-3BC7B4965104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>MUNICIPIO</t>
   </si>
@@ -44,15 +44,15 @@
     <t>UF</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>Indaiatuba</t>
   </si>
   <si>
     <t>SP</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Cariacica</t>
   </si>
   <si>
@@ -77,13 +77,10 @@
     <t>PR</t>
   </si>
   <si>
-    <t>Goiania</t>
+    <t>Jaguarão</t>
   </si>
   <si>
     <t>GO</t>
-  </si>
-  <si>
-    <t>Homologado</t>
   </si>
 </sst>
 </file>
@@ -433,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F94F8346-9FA2-4E48-83DE-F91F84112283}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -441,81 +438,78 @@
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
-        <v>15</v>
+      <c r="D3" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
-        <v>15</v>
+      <c r="D4" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
-        <v>15</v>
+      <c r="D5" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" t="s">
-        <v>15</v>
+      <c r="D6" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" t="s">
-        <v>15</v>
+      <c r="D7" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -525,6 +519,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="215e5025-edab-4c5b-b3d1-eab2d8030bb6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="558ba236-2e5d-4df0-8c7f-b30079445011" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F2B3038137E8F14588DFFF8123E7DA62" ma:contentTypeVersion="17" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="023335791d609f37f6f32b9e6d187ddb">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="215e5025-edab-4c5b-b3d1-eab2d8030bb6" xmlns:ns3="558ba236-2e5d-4df0-8c7f-b30079445011" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="14224507f95c74f5c8a044a57b33651f" ns2:_="" ns3:_="">
     <xsd:import namespace="215e5025-edab-4c5b-b3d1-eab2d8030bb6"/>
@@ -773,17 +778,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="215e5025-edab-4c5b-b3d1-eab2d8030bb6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="558ba236-2e5d-4df0-8c7f-b30079445011" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -794,6 +788,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D7A79FA-0280-4B97-9562-9B412635B81C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="215e5025-edab-4c5b-b3d1-eab2d8030bb6"/>
+    <ds:schemaRef ds:uri="558ba236-2e5d-4df0-8c7f-b30079445011"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3BDA35E3-8343-487E-80DC-EC374621626D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -812,17 +817,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D7A79FA-0280-4B97-9562-9B412635B81C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="215e5025-edab-4c5b-b3d1-eab2d8030bb6"/>
-    <ds:schemaRef ds:uri="558ba236-2e5d-4df0-8c7f-b30079445011"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FBB33F3-96AD-4679-872E-DD3B238C2E08}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
V2.1 - Ajustes e adição da coluna NfseNacional
</commit_message>
<xml_diff>
--- a/Cliente.xlsx
+++ b/Cliente.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source\MunicipiosHomologados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61568E3E-FA53-4723-89FF-3BC7B4965104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E16A371-9001-4600-B6BA-398A7F2F8D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
   <si>
     <t>MUNICIPIO</t>
   </si>
@@ -81,6 +81,15 @@
   </si>
   <si>
     <t>GO</t>
+  </si>
+  <si>
+    <t>Montezuma</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>Jequitaí</t>
   </si>
 </sst>
 </file>
@@ -430,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F94F8346-9FA2-4E48-83DE-F91F84112283}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -512,6 +521,22 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -519,14 +544,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="215e5025-edab-4c5b-b3d1-eab2d8030bb6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="558ba236-2e5d-4df0-8c7f-b30079445011" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -779,21 +802,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="215e5025-edab-4c5b-b3d1-eab2d8030bb6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="558ba236-2e5d-4df0-8c7f-b30079445011" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D7A79FA-0280-4B97-9562-9B412635B81C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FBB33F3-96AD-4679-872E-DD3B238C2E08}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="215e5025-edab-4c5b-b3d1-eab2d8030bb6"/>
-    <ds:schemaRef ds:uri="558ba236-2e5d-4df0-8c7f-b30079445011"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -818,9 +840,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FBB33F3-96AD-4679-872E-DD3B238C2E08}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D7A79FA-0280-4B97-9562-9B412635B81C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="215e5025-edab-4c5b-b3d1-eab2d8030bb6"/>
+    <ds:schemaRef ds:uri="558ba236-2e5d-4df0-8c7f-b30079445011"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
V2.2 - Melhoras no visual da planilha
</commit_message>
<xml_diff>
--- a/Cliente.xlsx
+++ b/Cliente.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source\MunicipiosHomologados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E16A371-9001-4600-B6BA-398A7F2F8D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF5D3EA-2325-4D1F-BC36-EFCA431C1C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
     <t>MUNICIPIO</t>
   </si>
@@ -90,6 +90,12 @@
   </si>
   <si>
     <t>Jequitaí</t>
+  </si>
+  <si>
+    <t>Anita Garibaldi</t>
+  </si>
+  <si>
+    <t>SC</t>
   </si>
 </sst>
 </file>
@@ -439,7 +445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F94F8346-9FA2-4E48-83DE-F91F84112283}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -537,6 +543,14 @@
         <v>16</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -544,15 +558,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F2B3038137E8F14588DFFF8123E7DA62" ma:contentTypeVersion="17" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="023335791d609f37f6f32b9e6d187ddb">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="215e5025-edab-4c5b-b3d1-eab2d8030bb6" xmlns:ns3="558ba236-2e5d-4df0-8c7f-b30079445011" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="14224507f95c74f5c8a044a57b33651f" ns2:_="" ns3:_="">
     <xsd:import namespace="215e5025-edab-4c5b-b3d1-eab2d8030bb6"/>
@@ -801,6 +806,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -813,14 +827,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FBB33F3-96AD-4679-872E-DD3B238C2E08}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3BDA35E3-8343-487E-80DC-EC374621626D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -839,6 +845,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FBB33F3-96AD-4679-872E-DD3B238C2E08}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D7A79FA-0280-4B97-9562-9B412635B81C}">
   <ds:schemaRefs>

</xml_diff>